<commit_message>
Added asinged tasks for Risk Register
</commit_message>
<xml_diff>
--- a/Iteration 3/Risk-Register.xlsx
+++ b/Iteration 3/Risk-Register.xlsx
@@ -5,12 +5,12 @@
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sara\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://temahau-my.sharepoint.com/personal/scatta1_student_eit_ac_nz/Documents/Desktop/AgileProject/AgileProjects_Repository/Iteration 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A2F9314-DDDE-456B-86E7-E230A005C34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{8A2F9314-DDDE-456B-86E7-E230A005C34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB5B4AB0-45D7-46E4-9F4E-BC1C79CA81CE}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example risk register" sheetId="8" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="107">
   <si>
     <t>REF ID</t>
   </si>
@@ -326,6 +326,78 @@
   <si>
     <t xml:space="preserve"> Syncing Git Repository Issues</t>
   </si>
+  <si>
+    <t xml:space="preserve">Miscomminication with goals for project </t>
+  </si>
+  <si>
+    <t>Commincation of the goals and deliverables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If communication isnt done effectively  </t>
+  </si>
+  <si>
+    <t>Formally plan future comminication in detail</t>
+  </si>
+  <si>
+    <t>No issues present/Under monitoring</t>
+  </si>
+  <si>
+    <t>unautherised access to project files and data</t>
+  </si>
+  <si>
+    <t>Members reciveing phising emails/messages</t>
+  </si>
+  <si>
+    <t>Members fall for phising emails/messages</t>
+  </si>
+  <si>
+    <t>No issues found/training project members</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report and recover data and train members </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full stack developer resigning </t>
+  </si>
+  <si>
+    <t>difficult development stages/any time</t>
+  </si>
+  <si>
+    <t>asinging big work loads to developer</t>
+  </si>
+  <si>
+    <t>hire a new developer/break up work laods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No issues/ under monitoring </t>
+  </si>
+  <si>
+    <t>Project Manager</t>
+  </si>
+  <si>
+    <t>Legal councel, Project manager</t>
+  </si>
+  <si>
+    <t>Commincations manager, PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> scheduling isnt cleary defined for goals and deliverables</t>
+  </si>
+  <si>
+    <t>when scheduling a project or deliverable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">incorrect scheduling information </t>
+  </si>
+  <si>
+    <t>diagnose causes, adjust scheduling accordingly, stronger communication</t>
+  </si>
+  <si>
+    <t>Closly monitoring with no errors found</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project monitoring </t>
+  </si>
 </sst>
 </file>
 
@@ -335,7 +407,7 @@
     <numFmt numFmtId="164" formatCode="mm/dd/yy;@"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -461,6 +533,18 @@
       <color theme="1"/>
       <name val="Century Gothic"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7.4"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="23">
@@ -692,7 +776,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
@@ -881,11 +965,17 @@
     <xf numFmtId="0" fontId="2" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1746,26 +1836,26 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:IW27"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="3.375" customWidth="1"/>
+    <col min="2" max="2" width="10.875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" style="5" customWidth="1"/>
     <col min="4" max="4" width="13.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="20.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="25.83203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="3.33203125" customWidth="1"/>
+    <col min="6" max="6" width="12.875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20.875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="25.875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15.875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12.875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="20.875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="3.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:257" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:257" x14ac:dyDescent="0.25">
       <c r="B1"/>
       <c r="C1"/>
       <c r="D1"/>
@@ -1780,7 +1870,7 @@
       <c r="M1"/>
       <c r="N1"/>
     </row>
-    <row r="2" spans="1:257" s="46" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:257" s="46" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="47"/>
       <c r="B2" s="48" t="s">
         <v>76</v>
@@ -2041,7 +2131,7 @@
       <c r="IV2" s="47"/>
       <c r="IW2" s="47"/>
     </row>
-    <row r="3" spans="1:257" ht="139" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:257" ht="138.94999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="1"/>
       <c r="F3" s="1"/>
       <c r="K3"/>
@@ -2049,13 +2139,13 @@
       <c r="M3"/>
       <c r="N3"/>
     </row>
-    <row r="4" spans="1:257" ht="79" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:257" ht="78.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="63"/>
       <c r="C4"/>
-      <c r="D4" s="66" t="s">
+      <c r="D4" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="66"/>
+      <c r="E4" s="67"/>
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4" s="62" t="s">
@@ -2068,7 +2158,7 @@
       <c r="M4"/>
       <c r="N4"/>
     </row>
-    <row r="5" spans="1:257" s="4" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:257" s="4" customFormat="1" ht="54.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="49" t="s">
         <v>0</v>
@@ -2111,7 +2201,7 @@
       </c>
       <c r="O5" s="3"/>
     </row>
-    <row r="6" spans="1:257" ht="100" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:257" ht="108" x14ac:dyDescent="0.25">
       <c r="B6" s="53">
         <v>10001</v>
       </c>
@@ -2151,7 +2241,7 @@
       </c>
       <c r="N6" s="65"/>
     </row>
-    <row r="7" spans="1:257" ht="100" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:257" ht="121.5" x14ac:dyDescent="0.25">
       <c r="B7" s="55">
         <v>10002</v>
       </c>
@@ -2191,7 +2281,7 @@
       </c>
       <c r="N7" s="65"/>
     </row>
-    <row r="8" spans="1:257" ht="100" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:257" ht="108" x14ac:dyDescent="0.25">
       <c r="B8" s="55">
         <v>10003</v>
       </c>
@@ -2231,7 +2321,7 @@
       </c>
       <c r="N8" s="65"/>
     </row>
-    <row r="9" spans="1:257" ht="75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:257" ht="81" x14ac:dyDescent="0.25">
       <c r="B9" s="55">
         <v>10004</v>
       </c>
@@ -2271,7 +2361,7 @@
       </c>
       <c r="N9" s="65"/>
     </row>
-    <row r="10" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="55"/>
       <c r="C10" s="54"/>
       <c r="D10" s="39"/>
@@ -2293,7 +2383,7 @@
       <c r="M10" s="64"/>
       <c r="N10" s="65"/>
     </row>
-    <row r="11" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="55"/>
       <c r="C11" s="54"/>
       <c r="D11" s="39"/>
@@ -2315,7 +2405,7 @@
       <c r="M11" s="64"/>
       <c r="N11" s="65"/>
     </row>
-    <row r="12" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="55"/>
       <c r="C12" s="54"/>
       <c r="D12" s="39"/>
@@ -2337,7 +2427,7 @@
       <c r="M12" s="64"/>
       <c r="N12" s="65"/>
     </row>
-    <row r="13" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="55"/>
       <c r="C13" s="54"/>
       <c r="D13" s="39"/>
@@ -2359,7 +2449,7 @@
       <c r="M13" s="64"/>
       <c r="N13" s="65"/>
     </row>
-    <row r="14" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="55"/>
       <c r="C14" s="54"/>
       <c r="D14" s="39"/>
@@ -2381,7 +2471,7 @@
       <c r="M14" s="64"/>
       <c r="N14" s="65"/>
     </row>
-    <row r="15" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="55"/>
       <c r="C15" s="54"/>
       <c r="D15" s="39"/>
@@ -2403,7 +2493,7 @@
       <c r="M15" s="64"/>
       <c r="N15" s="65"/>
     </row>
-    <row r="16" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="55"/>
       <c r="C16" s="54"/>
       <c r="D16" s="39"/>
@@ -2425,7 +2515,7 @@
       <c r="M16" s="64"/>
       <c r="N16" s="65"/>
     </row>
-    <row r="17" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="55"/>
       <c r="C17" s="54"/>
       <c r="D17" s="39"/>
@@ -2447,7 +2537,7 @@
       <c r="M17" s="64"/>
       <c r="N17" s="65"/>
     </row>
-    <row r="18" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="55"/>
       <c r="C18" s="54"/>
       <c r="D18" s="39"/>
@@ -2469,15 +2559,15 @@
       <c r="M18" s="64"/>
       <c r="N18" s="65"/>
     </row>
-    <row r="19" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="20" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="21" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="22" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="23" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="24" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="25" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D4:E4"/>
@@ -2575,23 +2665,23 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:IW43"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="3.375" customWidth="1"/>
+    <col min="2" max="2" width="10.875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.875" style="5" customWidth="1"/>
     <col min="4" max="4" width="13.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="29.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" style="1" customWidth="1"/>
-    <col min="9" max="12" width="15.83203125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="20.83203125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="3.33203125" customWidth="1"/>
+    <col min="5" max="5" width="29.375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="12.875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.875" style="1" customWidth="1"/>
+    <col min="9" max="12" width="15.875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12.875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="20.875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="3.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:257" s="46" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:257" s="46" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="47"/>
       <c r="B1" s="48" t="s">
         <v>77</v>
@@ -2852,7 +2942,7 @@
       <c r="IV1" s="47"/>
       <c r="IW1" s="47"/>
     </row>
-    <row r="2" spans="1:257" ht="139" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:257" ht="138.94999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C2" s="1"/>
       <c r="F2" s="1"/>
       <c r="K2"/>
@@ -2860,13 +2950,13 @@
       <c r="M2"/>
       <c r="N2"/>
     </row>
-    <row r="3" spans="1:257" ht="79" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:257" ht="78.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="63"/>
       <c r="C3"/>
-      <c r="D3" s="66" t="s">
+      <c r="D3" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="66"/>
+      <c r="E3" s="67"/>
       <c r="F3"/>
       <c r="G3"/>
       <c r="H3" s="62" t="s">
@@ -2879,7 +2969,7 @@
       <c r="M3"/>
       <c r="N3"/>
     </row>
-    <row r="4" spans="1:257" s="4" customFormat="1" ht="55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:257" s="4" customFormat="1" ht="54.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
       <c r="B4" s="49" t="s">
         <v>0</v>
@@ -2922,11 +3012,11 @@
       </c>
       <c r="O4" s="3"/>
     </row>
-    <row r="5" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="53">
         <v>1</v>
       </c>
-      <c r="C5" s="67">
+      <c r="C5" s="66">
         <v>46154</v>
       </c>
       <c r="D5" s="39"/>
@@ -2956,7 +3046,7 @@
       </c>
       <c r="N5" s="59"/>
     </row>
-    <row r="6" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="55"/>
       <c r="C6" s="54"/>
       <c r="D6" s="39"/>
@@ -2978,79 +3068,153 @@
       <c r="M6" s="6"/>
       <c r="N6" s="59"/>
     </row>
-    <row r="7" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="55"/>
-      <c r="C7" s="54"/>
+    <row r="7" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="55">
+        <v>3</v>
+      </c>
+      <c r="C7" s="54">
+        <v>46155</v>
+      </c>
       <c r="D7" s="39"/>
-      <c r="E7" s="61"/>
-      <c r="F7" s="56"/>
-      <c r="G7" s="57"/>
+      <c r="E7" s="61" t="s">
+        <v>83</v>
+      </c>
+      <c r="F7" s="56">
+        <v>2</v>
+      </c>
+      <c r="G7" s="57">
+        <v>8</v>
+      </c>
       <c r="H7" s="58">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
-      <c r="K7" s="61"/>
-      <c r="L7" s="61"/>
-      <c r="M7" s="6"/>
+        <v>16</v>
+      </c>
+      <c r="I7" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="J7" s="61" t="s">
+        <v>85</v>
+      </c>
+      <c r="K7" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="L7" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>100</v>
+      </c>
       <c r="N7" s="59"/>
     </row>
-    <row r="8" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="55"/>
+    <row r="8" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="55">
+        <v>4</v>
+      </c>
       <c r="C8" s="54"/>
       <c r="D8" s="39"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="56"/>
-      <c r="G8" s="57"/>
+      <c r="E8" s="61" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="56">
+        <v>5</v>
+      </c>
+      <c r="G8" s="57">
+        <v>16</v>
+      </c>
       <c r="H8" s="58">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="6"/>
+        <v>80</v>
+      </c>
+      <c r="I8" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="J8" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="K8" s="68" t="s">
+        <v>92</v>
+      </c>
+      <c r="L8" s="61" t="s">
+        <v>91</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>99</v>
+      </c>
       <c r="N8" s="59"/>
     </row>
-    <row r="9" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="55"/>
+    <row r="9" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="55">
+        <v>5</v>
+      </c>
       <c r="C9" s="54"/>
       <c r="D9" s="39"/>
-      <c r="E9" s="61"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="57"/>
+      <c r="E9" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="56">
+        <v>2</v>
+      </c>
+      <c r="G9" s="57">
+        <v>8</v>
+      </c>
       <c r="H9" s="58">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I9" s="61"/>
-      <c r="J9" s="61"/>
-      <c r="K9" s="61"/>
-      <c r="L9" s="61"/>
-      <c r="M9" s="6"/>
+        <v>16</v>
+      </c>
+      <c r="I9" s="61" t="s">
+        <v>94</v>
+      </c>
+      <c r="J9" s="61" t="s">
+        <v>95</v>
+      </c>
+      <c r="K9" s="61" t="s">
+        <v>96</v>
+      </c>
+      <c r="L9" s="61" t="s">
+        <v>97</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>98</v>
+      </c>
       <c r="N9" s="59"/>
     </row>
-    <row r="10" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="55"/>
+    <row r="10" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="55">
+        <v>6</v>
+      </c>
       <c r="C10" s="54"/>
       <c r="D10" s="39"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="57"/>
+      <c r="E10" s="61" t="s">
+        <v>101</v>
+      </c>
+      <c r="F10" s="56">
+        <v>3</v>
+      </c>
+      <c r="G10" s="57">
+        <v>16</v>
+      </c>
       <c r="H10" s="58">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I10" s="61"/>
-      <c r="J10" s="61"/>
-      <c r="K10" s="61"/>
-      <c r="L10" s="61"/>
-      <c r="M10" s="6"/>
+        <v>48</v>
+      </c>
+      <c r="I10" s="61" t="s">
+        <v>102</v>
+      </c>
+      <c r="J10" s="61" t="s">
+        <v>103</v>
+      </c>
+      <c r="K10" s="69" t="s">
+        <v>104</v>
+      </c>
+      <c r="L10" s="61" t="s">
+        <v>105</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>106</v>
+      </c>
       <c r="N10" s="59"/>
     </row>
-    <row r="11" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="55"/>
       <c r="C11" s="54"/>
       <c r="D11" s="39"/>
@@ -3068,7 +3232,7 @@
       <c r="M11" s="6"/>
       <c r="N11" s="59"/>
     </row>
-    <row r="12" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="55"/>
       <c r="C12" s="54"/>
       <c r="D12" s="39"/>
@@ -3086,7 +3250,7 @@
       <c r="M12" s="6"/>
       <c r="N12" s="59"/>
     </row>
-    <row r="13" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="55"/>
       <c r="C13" s="54"/>
       <c r="D13" s="39"/>
@@ -3104,7 +3268,7 @@
       <c r="M13" s="6"/>
       <c r="N13" s="59"/>
     </row>
-    <row r="14" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="55"/>
       <c r="C14" s="54"/>
       <c r="D14" s="39"/>
@@ -3122,7 +3286,7 @@
       <c r="M14" s="6"/>
       <c r="N14" s="59"/>
     </row>
-    <row r="15" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="55"/>
       <c r="C15" s="54"/>
       <c r="D15" s="39"/>
@@ -3140,7 +3304,7 @@
       <c r="M15" s="6"/>
       <c r="N15" s="59"/>
     </row>
-    <row r="16" spans="1:257" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:257" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="55"/>
       <c r="C16" s="54"/>
       <c r="D16" s="39"/>
@@ -3158,7 +3322,7 @@
       <c r="M16" s="6"/>
       <c r="N16" s="59"/>
     </row>
-    <row r="17" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="55"/>
       <c r="C17" s="54"/>
       <c r="D17" s="39"/>
@@ -3176,7 +3340,7 @@
       <c r="M17" s="6"/>
       <c r="N17" s="59"/>
     </row>
-    <row r="18" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="55"/>
       <c r="C18" s="54"/>
       <c r="D18" s="39"/>
@@ -3194,7 +3358,7 @@
       <c r="M18" s="6"/>
       <c r="N18" s="59"/>
     </row>
-    <row r="19" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="55"/>
       <c r="C19" s="54"/>
       <c r="D19" s="39"/>
@@ -3212,7 +3376,7 @@
       <c r="M19" s="6"/>
       <c r="N19" s="59"/>
     </row>
-    <row r="20" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="55"/>
       <c r="C20" s="54"/>
       <c r="D20" s="39"/>
@@ -3230,7 +3394,7 @@
       <c r="M20" s="6"/>
       <c r="N20" s="59"/>
     </row>
-    <row r="21" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="55"/>
       <c r="C21" s="54"/>
       <c r="D21" s="39"/>
@@ -3248,7 +3412,7 @@
       <c r="M21" s="6"/>
       <c r="N21" s="59"/>
     </row>
-    <row r="22" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="55"/>
       <c r="C22" s="54"/>
       <c r="D22" s="39"/>
@@ -3266,7 +3430,7 @@
       <c r="M22" s="6"/>
       <c r="N22" s="59"/>
     </row>
-    <row r="23" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="55"/>
       <c r="C23" s="54"/>
       <c r="D23" s="39"/>
@@ -3284,7 +3448,7 @@
       <c r="M23" s="6"/>
       <c r="N23" s="59"/>
     </row>
-    <row r="24" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="55"/>
       <c r="C24" s="54"/>
       <c r="D24" s="39"/>
@@ -3302,7 +3466,7 @@
       <c r="M24" s="6"/>
       <c r="N24" s="59"/>
     </row>
-    <row r="25" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="55"/>
       <c r="C25" s="54"/>
       <c r="D25" s="39"/>
@@ -3320,7 +3484,7 @@
       <c r="M25" s="6"/>
       <c r="N25" s="59"/>
     </row>
-    <row r="26" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="55"/>
       <c r="C26" s="54"/>
       <c r="D26" s="39"/>
@@ -3338,7 +3502,7 @@
       <c r="M26" s="6"/>
       <c r="N26" s="59"/>
     </row>
-    <row r="27" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="55"/>
       <c r="C27" s="54"/>
       <c r="D27" s="39"/>
@@ -3356,7 +3520,7 @@
       <c r="M27" s="6"/>
       <c r="N27" s="59"/>
     </row>
-    <row r="28" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="55"/>
       <c r="C28" s="54"/>
       <c r="D28" s="39"/>
@@ -3374,7 +3538,7 @@
       <c r="M28" s="6"/>
       <c r="N28" s="59"/>
     </row>
-    <row r="29" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="55"/>
       <c r="C29" s="54"/>
       <c r="D29" s="39"/>
@@ -3392,7 +3556,7 @@
       <c r="M29" s="6"/>
       <c r="N29" s="59"/>
     </row>
-    <row r="30" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="55"/>
       <c r="C30" s="54"/>
       <c r="D30" s="39"/>
@@ -3410,7 +3574,7 @@
       <c r="M30" s="6"/>
       <c r="N30" s="59"/>
     </row>
-    <row r="31" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="55"/>
       <c r="C31" s="54"/>
       <c r="D31" s="39"/>
@@ -3428,7 +3592,7 @@
       <c r="M31" s="6"/>
       <c r="N31" s="59"/>
     </row>
-    <row r="32" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="55"/>
       <c r="C32" s="54"/>
       <c r="D32" s="39"/>
@@ -3446,7 +3610,7 @@
       <c r="M32" s="6"/>
       <c r="N32" s="59"/>
     </row>
-    <row r="33" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="55"/>
       <c r="C33" s="54"/>
       <c r="D33" s="39"/>
@@ -3464,7 +3628,7 @@
       <c r="M33" s="6"/>
       <c r="N33" s="59"/>
     </row>
-    <row r="34" spans="2:14" ht="50.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="55"/>
       <c r="C34" s="54"/>
       <c r="D34" s="39"/>
@@ -3482,15 +3646,15 @@
       <c r="M34" s="6"/>
       <c r="N34" s="59"/>
     </row>
-    <row r="35" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="36" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="37" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="38" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="40" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="41" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="42" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="43" spans="2:14" ht="16" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="35" spans="2:14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="2:14" ht="15.95" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="D3:E3"/>
@@ -3587,21 +3751,21 @@
     <tabColor theme="2" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:IX27"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" customWidth="1"/>
-    <col min="2" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="3.33203125" customWidth="1"/>
+    <col min="1" max="1" width="3.375" customWidth="1"/>
+    <col min="2" max="4" width="22.875" customWidth="1"/>
+    <col min="5" max="5" width="3.375" customWidth="1"/>
     <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="7" max="7" width="3.33203125" customWidth="1"/>
+    <col min="7" max="7" width="3.375" customWidth="1"/>
     <col min="13" max="13" width="6.5" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" customWidth="1"/>
-    <col min="15" max="15" width="3.33203125" customWidth="1"/>
-    <col min="16" max="16" width="19.83203125" customWidth="1"/>
-    <col min="17" max="17" width="3.33203125" customWidth="1"/>
+    <col min="14" max="14" width="19.875" customWidth="1"/>
+    <col min="15" max="15" width="3.375" customWidth="1"/>
+    <col min="16" max="16" width="19.875" customWidth="1"/>
+    <col min="17" max="17" width="3.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:258" s="46" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:258" s="46" customFormat="1" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="47"/>
       <c r="B1" s="48" t="s">
         <v>27</v>
@@ -3863,7 +4027,7 @@
       <c r="IW1" s="47"/>
       <c r="IX1" s="47"/>
     </row>
-    <row r="2" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="45" t="s">
         <v>26</v>
       </c>
@@ -3893,7 +4057,7 @@
       <c r="M2" s="43"/>
       <c r="O2" s="42"/>
     </row>
-    <row r="3" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="40" t="s">
         <v>21</v>
       </c>
@@ -3930,7 +4094,7 @@
       <c r="M3" s="2"/>
       <c r="O3" s="19"/>
     </row>
-    <row r="4" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="35" t="s">
         <v>18</v>
       </c>
@@ -3967,7 +4131,7 @@
       <c r="M4" s="2"/>
       <c r="O4" s="19"/>
     </row>
-    <row r="5" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="29" t="s">
         <v>15</v>
       </c>
@@ -4004,7 +4168,7 @@
       <c r="M5" s="2"/>
       <c r="O5" s="19"/>
     </row>
-    <row r="6" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="24" t="s">
         <v>12</v>
       </c>
@@ -4041,7 +4205,7 @@
       <c r="M6" s="2"/>
       <c r="O6" s="19"/>
     </row>
-    <row r="7" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="17" t="s">
         <v>9</v>
       </c>
@@ -4076,7 +4240,7 @@
       </c>
       <c r="O7" s="10"/>
     </row>
-    <row r="8" spans="1:258" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:258" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -4084,7 +4248,7 @@
       <c r="K8" s="8"/>
       <c r="L8" s="8"/>
     </row>
-    <row r="9" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="41" t="s">
         <v>23</v>
       </c>
@@ -4092,7 +4256,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="37">
         <v>1</v>
       </c>
@@ -4100,7 +4264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="31">
         <v>2</v>
       </c>
@@ -4108,7 +4272,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="26">
         <v>3</v>
       </c>
@@ -4116,7 +4280,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="20">
         <v>4</v>
       </c>
@@ -4124,7 +4288,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:258" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:258" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="11">
         <v>5</v>
       </c>
@@ -4132,62 +4296,62 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:258" ht="44.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:258" ht="44.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="63" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="45" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="60" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="60" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="60" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="60" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="60" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="60" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="24" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="60" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="60" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="60" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="2:2" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="60" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Changed Test Plan Matrix
</commit_message>
<xml_diff>
--- a/Iteration 3/Risk-Register.xlsx
+++ b/Iteration 3/Risk-Register.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b444fedf9e291051/Desktop/AgileProjects_Repository/Iteration 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="191" documentId="13_ncr:1_{8A2F9314-DDDE-456B-86E7-E230A005C34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44FB3796-F048-49BB-8322-EF594F485D81}"/>
+  <xr:revisionPtr revIDLastSave="195" documentId="13_ncr:1_{8A2F9314-DDDE-456B-86E7-E230A005C34E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C17150BE-4FED-4D5D-BF25-039141873156}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="145">
   <si>
     <t>REF ID</t>
   </si>
@@ -502,6 +502,15 @@
   </si>
   <si>
     <t>internet connection problems may disturb development work</t>
+  </si>
+  <si>
+    <t>wifi cuts off/powercut due to bad weather</t>
+  </si>
+  <si>
+    <t>ensure work is saved frequently and keep offline copies of important files</t>
+  </si>
+  <si>
+    <t>no issues as of present</t>
   </si>
 </sst>
 </file>
@@ -3566,10 +3575,18 @@
       <c r="I16" s="61" t="s">
         <v>124</v>
       </c>
-      <c r="J16" s="61"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="6"/>
+      <c r="J16" s="61" t="s">
+        <v>142</v>
+      </c>
+      <c r="K16" s="61" t="s">
+        <v>143</v>
+      </c>
+      <c r="L16" s="61" t="s">
+        <v>144</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>129</v>
+      </c>
       <c r="N16" s="59"/>
     </row>
     <row r="17" spans="2:14" ht="50.1" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>